<commit_message>
feat: Excel入力対応 + clean_name改善
- scraper_dermatology.py: input.xlsx (A列) からキーワードを読み込み、
  キーワード1件につき上位1URL を収集して output_*.xlsx に出力
- clean_name: 皮ふ科（ひらがな）をCLINIC_KEYWORDSに追加
- clean_name: キーワードで始まる汎用セグメント（皮膚科専門医院等）を-3点減点して
  固有名詞を持つ正しいクリニック名を優先選択（全19テストケースパス）
- .gitignore: output_*.xlsx パターンを追加
- input.xlsx: サンプルキーワード3件（埼玉県皮膚科）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -419,28 +419,28 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>検索キーワード</t>
+          <t>キーワード</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>スターバックス 新宿</t>
+          <t>さいたま市 皮膚科 クリニック</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ユニクロ 渋谷</t>
+          <t>川越市 皮膚科</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>マクドナルド 銀座</t>
+          <t>越谷市 皮膚科 クリニック</t>
         </is>
       </c>
     </row>

</xml_diff>